<commit_message>
Geoportal: mejorar ficha institucional y refrescar interfaz
</commit_message>
<xml_diff>
--- a/docs/descargas/cobertura_mapeo_osm.xlsx
+++ b/docs/descargas/cobertura_mapeo_osm.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" r:id="Rfa3b264c589441e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="2" r:id="R252066660a00493b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Año 2026" sheetId="3" r:id="R7831640195934963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" r:id="R47e5d6e48a234e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="2" r:id="Ra01d281a32bf4559"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Año 2026" sheetId="3" r:id="R850802f8c2f840c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -557,7 +557,7 @@
         <x:v>Producto</x:v>
       </x:c>
       <x:c r="B4" s="7" t="str">
-        <x:v>Descarga pública del Catálogo de datos del Observatorio REDSA</x:v>
+        <x:v>Descarga pública del Catálogo de datos del Observatorio de Seguridad Vial y Movilidad Sostenible</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>

<commit_message>
feat: ampliar serie territorial ANT e INEC hasta 2026
</commit_message>
<xml_diff>
--- a/docs/descargas/cobertura_mapeo_osm.xlsx
+++ b/docs/descargas/cobertura_mapeo_osm.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" r:id="R47e5d6e48a234e82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="2" r:id="Ra01d281a32bf4559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Año 2026" sheetId="3" r:id="R850802f8c2f840c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" r:id="R2733f6d88c984e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodología" sheetId="2" r:id="Re504afa6c0f04ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Año 2026" sheetId="3" r:id="Raf8ae43ce691468a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -243,7 +243,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -308,22 +308,34 @@
     <x:xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="6" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="6" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="6" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="7" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="7" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="7" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -613,7 +625,7 @@
         <x:v>Generado</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>2026-07-27</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -629,7 +641,7 @@
         <x:v>Cómo leer</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
-        <x:v>Cada hoja anual presenta total nacional, subtotales provinciales y datos cantonales. Cuando existe nivel parroquial, incluye además subtotales cantonales y el detalle parroquial.</x:v>
+        <x:v>Cada hoja anual usa el nivel más detallado realmente disponible: parroquia cuando existe información comprobable para ese año; en caso contrario, cantón o provincia. Incluye subtotales y total nacional.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -645,7 +657,7 @@
         <x:v>Citación sugerida</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>Fundación REDSA (2026). Cobertura del mapeo de infraestructura vial. Observatorio Ciudadano de Seguridad Vial y Movilidad Sostenible. Consulta: 2026-07-22.</x:v>
+        <x:v>Fundación REDSA (2026). Cobertura del mapeo de infraestructura vial. Observatorio Ciudadano de Seguridad Vial y Movilidad Sostenible. Consulta: 2026-07-27.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -765,6 +777,7 @@
     <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="55" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -781,6 +794,7 @@
       <x:c r="I1" s="2"/>
       <x:c r="J1" s="2"/>
       <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2"/>
@@ -794,6 +808,7 @@
       <x:c r="I2" s="2"/>
       <x:c r="J2" s="2"/>
       <x:c r="K2" s="2"/>
+      <x:c r="L2" s="2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="12" t="str">
@@ -809,6 +824,7 @@
       <x:c r="I3" s="12"/>
       <x:c r="J3" s="12"/>
       <x:c r="K3" s="12"/>
+      <x:c r="L3" s="12"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="33" t="str">
@@ -841,8 +857,11 @@
       <x:c r="J5" s="34" t="str">
         <x:v>Numerador</x:v>
       </x:c>
-      <x:c r="K5" s="35" t="str">
+      <x:c r="K5" s="34" t="str">
         <x:v>Denominador</x:v>
+      </x:c>
+      <x:c r="L5" s="35" t="str">
+        <x:v>Observación</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -866,9 +885,10 @@
       <x:c r="J6" s="39" t="n">
         <x:v>40901</x:v>
       </x:c>
-      <x:c r="K6" s="40" t="n">
+      <x:c r="K6" s="39" t="n">
         <x:v>17966573</x:v>
       </x:c>
+      <x:c r="L6" s="56" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="41" t="str">
@@ -893,9 +913,10 @@
       <x:c r="J7" s="44" t="n">
         <x:v>6197</x:v>
       </x:c>
-      <x:c r="K7" s="45" t="n">
+      <x:c r="K7" s="44" t="n">
         <x:v>831220</x:v>
       </x:c>
+      <x:c r="L7" s="57" t="str"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="46" t="str">
@@ -924,9 +945,10 @@
       <x:c r="J8" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K8" s="50" t="n">
+      <x:c r="K8" s="49" t="n">
         <x:v>24624</x:v>
       </x:c>
+      <x:c r="L8" s="58" t="str"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="46" t="str">
@@ -955,9 +977,10 @@
       <x:c r="J9" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K9" s="50" t="n">
+      <x:c r="K9" s="49" t="n">
         <x:v>12432</x:v>
       </x:c>
+      <x:c r="L9" s="58" t="str"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="46" t="str">
@@ -986,9 +1009,10 @@
       <x:c r="J10" s="49" t="n">
         <x:v>6065</x:v>
       </x:c>
-      <x:c r="K10" s="50" t="n">
+      <x:c r="K10" s="49" t="n">
         <x:v>619701</x:v>
       </x:c>
+      <x:c r="L10" s="58" t="str"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="46" t="str">
@@ -1017,9 +1041,10 @@
       <x:c r="J11" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K11" s="50" t="n">
+      <x:c r="K11" s="49" t="n">
         <x:v>2779</x:v>
       </x:c>
+      <x:c r="L11" s="58" t="str"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="46" t="str">
@@ -1048,9 +1073,10 @@
       <x:c r="J12" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K12" s="50" t="n">
+      <x:c r="K12" s="49" t="n">
         <x:v>12492</x:v>
       </x:c>
+      <x:c r="L12" s="58" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="46" t="str">
@@ -1079,9 +1105,10 @@
       <x:c r="J13" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K13" s="50" t="n">
+      <x:c r="K13" s="49" t="n">
         <x:v>3648</x:v>
       </x:c>
+      <x:c r="L13" s="58" t="str"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="46" t="str">
@@ -1110,9 +1137,10 @@
       <x:c r="J14" s="49" t="n">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="K14" s="50" t="n">
+      <x:c r="K14" s="49" t="n">
         <x:v>44577</x:v>
       </x:c>
+      <x:c r="L14" s="58" t="str"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="46" t="str">
@@ -1141,9 +1169,10 @@
       <x:c r="J15" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K15" s="50" t="n">
+      <x:c r="K15" s="49" t="n">
         <x:v>14972</x:v>
       </x:c>
+      <x:c r="L15" s="58" t="str"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="46" t="str">
@@ -1172,9 +1201,10 @@
       <x:c r="J16" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K16" s="50" t="n">
+      <x:c r="K16" s="49" t="n">
         <x:v>3503</x:v>
       </x:c>
+      <x:c r="L16" s="58" t="str"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="46" t="str">
@@ -1203,9 +1233,10 @@
       <x:c r="J17" s="49" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="K17" s="50" t="n">
+      <x:c r="K17" s="49" t="n">
         <x:v>27385</x:v>
       </x:c>
+      <x:c r="L17" s="58" t="str"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="46" t="str">
@@ -1234,9 +1265,10 @@
       <x:c r="J18" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K18" s="50" t="n">
+      <x:c r="K18" s="49" t="n">
         <x:v>9825</x:v>
       </x:c>
+      <x:c r="L18" s="58" t="str"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="46" t="str">
@@ -1265,9 +1297,10 @@
       <x:c r="J19" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K19" s="50" t="n">
+      <x:c r="K19" s="49" t="n">
         <x:v>3760</x:v>
       </x:c>
+      <x:c r="L19" s="58" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="46" t="str">
@@ -1296,9 +1329,10 @@
       <x:c r="J20" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K20" s="50" t="n">
+      <x:c r="K20" s="49" t="n">
         <x:v>20985</x:v>
       </x:c>
+      <x:c r="L20" s="58" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="46" t="str">
@@ -1327,9 +1361,10 @@
       <x:c r="J21" s="49" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K21" s="50" t="n">
+      <x:c r="K21" s="49" t="n">
         <x:v>4621</x:v>
       </x:c>
+      <x:c r="L21" s="58" t="str"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="46" t="str">
@@ -1358,9 +1393,10 @@
       <x:c r="J22" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K22" s="50" t="n">
+      <x:c r="K22" s="49" t="n">
         <x:v>25916</x:v>
       </x:c>
+      <x:c r="L22" s="58" t="str"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="41" t="str">
@@ -1385,9 +1421,10 @@
       <x:c r="J23" s="44" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="K23" s="45" t="n">
+      <x:c r="K23" s="44" t="n">
         <x:v>204410</x:v>
       </x:c>
+      <x:c r="L23" s="57" t="str"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="46" t="str">
@@ -1416,9 +1453,10 @@
       <x:c r="J24" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K24" s="50" t="n">
+      <x:c r="K24" s="49" t="n">
         <x:v>16429</x:v>
       </x:c>
+      <x:c r="L24" s="58" t="str"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="46" t="str">
@@ -1447,9 +1485,10 @@
       <x:c r="J25" s="49" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K25" s="50" t="n">
+      <x:c r="K25" s="49" t="n">
         <x:v>20223</x:v>
       </x:c>
+      <x:c r="L25" s="58" t="str"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="46" t="str">
@@ -1478,9 +1517,10 @@
       <x:c r="J26" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K26" s="50" t="n">
+      <x:c r="K26" s="49" t="n">
         <x:v>15659</x:v>
       </x:c>
+      <x:c r="L26" s="58" t="str"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="46" t="str">
@@ -1509,9 +1549,10 @@
       <x:c r="J27" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K27" s="50" t="n">
+      <x:c r="K27" s="49" t="n">
         <x:v>15434</x:v>
       </x:c>
+      <x:c r="L27" s="58" t="str"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="46" t="str">
@@ -1540,9 +1581,10 @@
       <x:c r="J28" s="49" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K28" s="50" t="n">
+      <x:c r="K28" s="49" t="n">
         <x:v>100508</x:v>
       </x:c>
+      <x:c r="L28" s="58" t="str"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="46" t="str">
@@ -1571,9 +1613,10 @@
       <x:c r="J29" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K29" s="50" t="n">
+      <x:c r="K29" s="49" t="n">
         <x:v>7297</x:v>
       </x:c>
+      <x:c r="L29" s="58" t="str"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="46" t="str">
@@ -1602,9 +1645,10 @@
       <x:c r="J30" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K30" s="50" t="n">
+      <x:c r="K30" s="49" t="n">
         <x:v>28860</x:v>
       </x:c>
+      <x:c r="L30" s="58" t="str"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="41" t="str">
@@ -1629,9 +1673,10 @@
       <x:c r="J31" s="44" t="n">
         <x:v>276</x:v>
       </x:c>
-      <x:c r="K31" s="45" t="n">
+      <x:c r="K31" s="44" t="n">
         <x:v>237470</x:v>
       </x:c>
+      <x:c r="L31" s="57" t="str"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="46" t="str">
@@ -1660,9 +1705,10 @@
       <x:c r="J32" s="49" t="n">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="K32" s="50" t="n">
+      <x:c r="K32" s="49" t="n">
         <x:v>77677</x:v>
       </x:c>
+      <x:c r="L32" s="58" t="str"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="46" t="str">
@@ -1691,9 +1737,10 @@
       <x:c r="J33" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K33" s="50" t="n">
+      <x:c r="K33" s="49" t="n">
         <x:v>18986</x:v>
       </x:c>
+      <x:c r="L33" s="58" t="str"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="46" t="str">
@@ -1722,9 +1769,10 @@
       <x:c r="J34" s="49" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="K34" s="50" t="n">
+      <x:c r="K34" s="49" t="n">
         <x:v>52602</x:v>
       </x:c>
+      <x:c r="L34" s="58" t="str"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="46" t="str">
@@ -1753,9 +1801,10 @@
       <x:c r="J35" s="49" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="K35" s="50" t="n">
+      <x:c r="K35" s="49" t="n">
         <x:v>6272</x:v>
       </x:c>
+      <x:c r="L35" s="58" t="str"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="46" t="str">
@@ -1784,9 +1833,10 @@
       <x:c r="J36" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K36" s="50" t="n">
+      <x:c r="K36" s="49" t="n">
         <x:v>9670</x:v>
       </x:c>
+      <x:c r="L36" s="58" t="str"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="46" t="str">
@@ -1815,9 +1865,10 @@
       <x:c r="J37" s="49" t="n">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="K37" s="50" t="n">
+      <x:c r="K37" s="49" t="n">
         <x:v>67598</x:v>
       </x:c>
+      <x:c r="L37" s="58" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="46" t="str">
@@ -1846,9 +1897,10 @@
       <x:c r="J38" s="49" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K38" s="50" t="n">
+      <x:c r="K38" s="49" t="n">
         <x:v>4665</x:v>
       </x:c>
+      <x:c r="L38" s="58" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="41" t="str">
@@ -1873,9 +1925,10 @@
       <x:c r="J39" s="44" t="n">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="K39" s="45" t="n">
+      <x:c r="K39" s="44" t="n">
         <x:v>177813</x:v>
       </x:c>
+      <x:c r="L39" s="57" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="46" t="str">
@@ -1904,9 +1957,10 @@
       <x:c r="J40" s="49" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="K40" s="50" t="n">
+      <x:c r="K40" s="49" t="n">
         <x:v>16366</x:v>
       </x:c>
+      <x:c r="L40" s="58" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="46" t="str">
@@ -1935,9 +1989,10 @@
       <x:c r="J41" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K41" s="50" t="n">
+      <x:c r="K41" s="49" t="n">
         <x:v>14669</x:v>
       </x:c>
+      <x:c r="L41" s="58" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="46" t="str">
@@ -1966,9 +2021,10 @@
       <x:c r="J42" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K42" s="50" t="n">
+      <x:c r="K42" s="49" t="n">
         <x:v>12935</x:v>
       </x:c>
+      <x:c r="L42" s="58" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="46" t="str">
@@ -1997,9 +2053,10 @@
       <x:c r="J43" s="49" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="K43" s="50" t="n">
+      <x:c r="K43" s="49" t="n">
         <x:v>30427</x:v>
       </x:c>
+      <x:c r="L43" s="58" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="46" t="str">
@@ -2028,9 +2085,10 @@
       <x:c r="J44" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K44" s="50" t="n">
+      <x:c r="K44" s="49" t="n">
         <x:v>7994</x:v>
       </x:c>
+      <x:c r="L44" s="58" t="str"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="46" t="str">
@@ -2059,9 +2117,10 @@
       <x:c r="J45" s="49" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K45" s="50" t="n">
+      <x:c r="K45" s="49" t="n">
         <x:v>95422</x:v>
       </x:c>
+      <x:c r="L45" s="58" t="str"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="41" t="str">
@@ -2086,9 +2145,10 @@
       <x:c r="J46" s="44" t="n">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="K46" s="45" t="n">
+      <x:c r="K46" s="44" t="n">
         <x:v>488857</x:v>
       </x:c>
+      <x:c r="L46" s="57" t="str"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="46" t="str">
@@ -2117,9 +2177,10 @@
       <x:c r="J47" s="49" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="K47" s="50" t="n">
+      <x:c r="K47" s="49" t="n">
         <x:v>38530</x:v>
       </x:c>
+      <x:c r="L47" s="58" t="str"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="46" t="str">
@@ -2148,9 +2209,10 @@
       <x:c r="J48" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K48" s="50" t="n">
+      <x:c r="K48" s="49" t="n">
         <x:v>13790</x:v>
       </x:c>
+      <x:c r="L48" s="58" t="str"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="46" t="str">
@@ -2179,9 +2241,10 @@
       <x:c r="J49" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K49" s="50" t="n">
+      <x:c r="K49" s="49" t="n">
         <x:v>10951</x:v>
       </x:c>
+      <x:c r="L49" s="58" t="str"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="46" t="str">
@@ -2210,9 +2273,10 @@
       <x:c r="J50" s="49" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K50" s="50" t="n">
+      <x:c r="K50" s="49" t="n">
         <x:v>30603</x:v>
       </x:c>
+      <x:c r="L50" s="58" t="str"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="46" t="str">
@@ -2241,9 +2305,10 @@
       <x:c r="J51" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K51" s="50" t="n">
+      <x:c r="K51" s="49" t="n">
         <x:v>17515</x:v>
       </x:c>
+      <x:c r="L51" s="58" t="str"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="46" t="str">
@@ -2272,9 +2337,10 @@
       <x:c r="J52" s="49" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K52" s="50" t="n">
+      <x:c r="K52" s="49" t="n">
         <x:v>36664</x:v>
       </x:c>
+      <x:c r="L52" s="58" t="str"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="46" t="str">
@@ -2303,9 +2369,10 @@
       <x:c r="J53" s="49" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="K53" s="50" t="n">
+      <x:c r="K53" s="49" t="n">
         <x:v>49466</x:v>
       </x:c>
+      <x:c r="L53" s="58" t="str"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="46" t="str">
@@ -2334,9 +2401,10 @@
       <x:c r="J54" s="49" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="K54" s="50" t="n">
+      <x:c r="K54" s="49" t="n">
         <x:v>12202</x:v>
       </x:c>
+      <x:c r="L54" s="58" t="str"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="46" t="str">
@@ -2365,9 +2433,10 @@
       <x:c r="J55" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K55" s="50" t="n">
+      <x:c r="K55" s="49" t="n">
         <x:v>6957</x:v>
       </x:c>
+      <x:c r="L55" s="58" t="str"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="46" t="str">
@@ -2396,9 +2465,10 @@
       <x:c r="J56" s="49" t="n">
         <x:v>329</x:v>
       </x:c>
-      <x:c r="K56" s="50" t="n">
+      <x:c r="K56" s="49" t="n">
         <x:v>272179</x:v>
       </x:c>
+      <x:c r="L56" s="58" t="str"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="41" t="str">
@@ -2423,9 +2493,10 @@
       <x:c r="J57" s="44" t="n">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="K57" s="45" t="n">
+      <x:c r="K57" s="44" t="n">
         <x:v>489147</x:v>
       </x:c>
+      <x:c r="L57" s="57" t="str"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="46" t="str">
@@ -2454,9 +2525,10 @@
       <x:c r="J58" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K58" s="50" t="n">
+      <x:c r="K58" s="49" t="n">
         <x:v>57161</x:v>
       </x:c>
+      <x:c r="L58" s="58" t="str"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="46" t="str">
@@ -2485,9 +2557,10 @@
       <x:c r="J59" s="49" t="n">
         <x:v>274</x:v>
       </x:c>
-      <x:c r="K59" s="50" t="n">
+      <x:c r="K59" s="49" t="n">
         <x:v>227737</x:v>
       </x:c>
+      <x:c r="L59" s="58" t="str"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="46" t="str">
@@ -2516,9 +2589,10 @@
       <x:c r="J60" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K60" s="50" t="n">
+      <x:c r="K60" s="49" t="n">
         <x:v>22602</x:v>
       </x:c>
+      <x:c r="L60" s="58" t="str"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="46" t="str">
@@ -2547,9 +2621,10 @@
       <x:c r="J61" s="49" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="K61" s="50" t="n">
+      <x:c r="K61" s="49" t="n">
         <x:v>68420</x:v>
       </x:c>
+      <x:c r="L61" s="58" t="str"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="46" t="str">
@@ -2578,9 +2653,10 @@
       <x:c r="J62" s="49" t="n">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="K62" s="50" t="n">
+      <x:c r="K62" s="49" t="n">
         <x:v>69816</x:v>
       </x:c>
+      <x:c r="L62" s="58" t="str"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="46" t="str">
@@ -2609,9 +2685,10 @@
       <x:c r="J63" s="49" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="K63" s="50" t="n">
+      <x:c r="K63" s="49" t="n">
         <x:v>24838</x:v>
       </x:c>
+      <x:c r="L63" s="58" t="str"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="46" t="str">
@@ -2640,9 +2717,10 @@
       <x:c r="J64" s="49" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="K64" s="50" t="n">
+      <x:c r="K64" s="49" t="n">
         <x:v>18573</x:v>
       </x:c>
+      <x:c r="L64" s="58" t="str"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="41" t="str">
@@ -2667,9 +2745,10 @@
       <x:c r="J65" s="44" t="n">
         <x:v>389</x:v>
       </x:c>
-      <x:c r="K65" s="45" t="n">
+      <x:c r="K65" s="44" t="n">
         <x:v>748627</x:v>
       </x:c>
+      <x:c r="L65" s="57" t="str"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="46" t="str">
@@ -2698,9 +2777,10 @@
       <x:c r="J66" s="49" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="K66" s="50" t="n">
+      <x:c r="K66" s="49" t="n">
         <x:v>33741</x:v>
       </x:c>
+      <x:c r="L66" s="58" t="str"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="46" t="str">
@@ -2729,9 +2809,10 @@
       <x:c r="J67" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K67" s="50" t="n">
+      <x:c r="K67" s="49" t="n">
         <x:v>6242</x:v>
       </x:c>
+      <x:c r="L67" s="58" t="str"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="46" t="str">
@@ -2760,9 +2841,10 @@
       <x:c r="J68" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K68" s="50" t="n">
+      <x:c r="K68" s="49" t="n">
         <x:v>8176</x:v>
       </x:c>
+      <x:c r="L68" s="58" t="str"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="46" t="str">
@@ -2791,9 +2873,10 @@
       <x:c r="J69" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K69" s="50" t="n">
+      <x:c r="K69" s="49" t="n">
         <x:v>2275</x:v>
       </x:c>
+      <x:c r="L69" s="58" t="str"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="46" t="str">
@@ -2822,9 +2905,10 @@
       <x:c r="J70" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K70" s="50" t="n">
+      <x:c r="K70" s="49" t="n">
         <x:v>63314</x:v>
       </x:c>
+      <x:c r="L70" s="58" t="str"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="46" t="str">
@@ -2853,9 +2937,10 @@
       <x:c r="J71" s="49" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="K71" s="50" t="n">
+      <x:c r="K71" s="49" t="n">
         <x:v>59696</x:v>
       </x:c>
+      <x:c r="L71" s="58" t="str"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="46" t="str">
@@ -2884,9 +2969,10 @@
       <x:c r="J72" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K72" s="50" t="n">
+      <x:c r="K72" s="49" t="n">
         <x:v>5902</x:v>
       </x:c>
+      <x:c r="L72" s="58" t="str"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="46" t="str">
@@ -2915,9 +3001,10 @@
       <x:c r="J73" s="49" t="n">
         <x:v>282</x:v>
       </x:c>
-      <x:c r="K73" s="50" t="n">
+      <x:c r="K73" s="49" t="n">
         <x:v>321196</x:v>
       </x:c>
+      <x:c r="L73" s="58" t="str"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="46" t="str">
@@ -2946,9 +3033,10 @@
       <x:c r="J74" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K74" s="50" t="n">
+      <x:c r="K74" s="49" t="n">
         <x:v>7090</x:v>
       </x:c>
+      <x:c r="L74" s="58" t="str"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="46" t="str">
@@ -2977,9 +3065,10 @@
       <x:c r="J75" s="49" t="n">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="K75" s="50" t="n">
+      <x:c r="K75" s="49" t="n">
         <x:v>86890</x:v>
       </x:c>
+      <x:c r="L75" s="58" t="str"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="46" t="str">
@@ -3008,9 +3097,10 @@
       <x:c r="J76" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K76" s="50" t="n">
+      <x:c r="K76" s="49" t="n">
         <x:v>30186</x:v>
       </x:c>
+      <x:c r="L76" s="58" t="str"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="46" t="str">
@@ -3039,9 +3129,10 @@
       <x:c r="J77" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K77" s="50" t="n">
+      <x:c r="K77" s="49" t="n">
         <x:v>14004</x:v>
       </x:c>
+      <x:c r="L77" s="58" t="str"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="46" t="str">
@@ -3070,9 +3161,10 @@
       <x:c r="J78" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K78" s="50" t="n">
+      <x:c r="K78" s="49" t="n">
         <x:v>84807</x:v>
       </x:c>
+      <x:c r="L78" s="58" t="str"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="46" t="str">
@@ -3101,9 +3193,10 @@
       <x:c r="J79" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K79" s="50" t="n">
+      <x:c r="K79" s="49" t="n">
         <x:v>25108</x:v>
       </x:c>
+      <x:c r="L79" s="58" t="str"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="41" t="str">
@@ -3128,9 +3221,10 @@
       <x:c r="J80" s="44" t="n">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="K80" s="45" t="n">
+      <x:c r="K80" s="44" t="n">
         <x:v>601626</x:v>
       </x:c>
+      <x:c r="L80" s="57" t="str"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="46" t="str">
@@ -3159,9 +3253,10 @@
       <x:c r="J81" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K81" s="50" t="n">
+      <x:c r="K81" s="49" t="n">
         <x:v>55418</x:v>
       </x:c>
+      <x:c r="L81" s="58" t="str"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="46" t="str">
@@ -3190,9 +3285,10 @@
       <x:c r="J82" s="49" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="K82" s="50" t="n">
+      <x:c r="K82" s="49" t="n">
         <x:v>51603</x:v>
       </x:c>
+      <x:c r="L82" s="58" t="str"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="46" t="str">
@@ -3221,9 +3317,10 @@
       <x:c r="J83" s="49" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="K83" s="50" t="n">
+      <x:c r="K83" s="49" t="n">
         <x:v>231097</x:v>
       </x:c>
+      <x:c r="L83" s="58" t="str"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="46" t="str">
@@ -3252,9 +3349,10 @@
       <x:c r="J84" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K84" s="50" t="n">
+      <x:c r="K84" s="49" t="n">
         <x:v>38495</x:v>
       </x:c>
+      <x:c r="L84" s="58" t="str"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="46" t="str">
@@ -3283,9 +3381,10 @@
       <x:c r="J85" s="49" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K85" s="50" t="n">
+      <x:c r="K85" s="49" t="n">
         <x:v>134059</x:v>
       </x:c>
+      <x:c r="L85" s="58" t="str"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="46" t="str">
@@ -3314,9 +3413,10 @@
       <x:c r="J86" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K86" s="50" t="n">
+      <x:c r="K86" s="49" t="n">
         <x:v>36052</x:v>
       </x:c>
+      <x:c r="L86" s="58" t="str"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="46" t="str">
@@ -3345,9 +3445,10 @@
       <x:c r="J87" s="49" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K87" s="50" t="n">
+      <x:c r="K87" s="49" t="n">
         <x:v>54902</x:v>
       </x:c>
+      <x:c r="L87" s="58" t="str"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="41" t="str">
@@ -3372,9 +3473,10 @@
       <x:c r="J88" s="44" t="n">
         <x:v>142</x:v>
       </x:c>
-      <x:c r="K88" s="45" t="n">
+      <x:c r="K88" s="44" t="n">
         <x:v>30082</x:v>
       </x:c>
+      <x:c r="L88" s="57" t="str"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="46" t="str">
@@ -3403,9 +3505,10 @@
       <x:c r="J89" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K89" s="50" t="n">
+      <x:c r="K89" s="49" t="n">
         <x:v>3205</x:v>
       </x:c>
+      <x:c r="L89" s="58" t="str"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="46" t="str">
@@ -3434,9 +3537,10 @@
       <x:c r="J90" s="49" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="K90" s="50" t="n">
+      <x:c r="K90" s="49" t="n">
         <x:v>8850</x:v>
       </x:c>
+      <x:c r="L90" s="58" t="str"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="46" t="str">
@@ -3465,9 +3569,10 @@
       <x:c r="J91" s="49" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="K91" s="50" t="n">
+      <x:c r="K91" s="49" t="n">
         <x:v>18027</x:v>
       </x:c>
+      <x:c r="L91" s="58" t="str"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="41" t="str">
@@ -3492,9 +3597,10 @@
       <x:c r="J92" s="44" t="n">
         <x:v>5333</x:v>
       </x:c>
-      <x:c r="K92" s="45" t="n">
+      <x:c r="K92" s="44" t="n">
         <x:v>4739771</x:v>
       </x:c>
+      <x:c r="L92" s="57" t="str"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="46" t="str">
@@ -3523,9 +3629,10 @@
       <x:c r="J93" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K93" s="50" t="n">
+      <x:c r="K93" s="49" t="n">
         <x:v>26556</x:v>
       </x:c>
+      <x:c r="L93" s="58" t="str"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="46" t="str">
@@ -3554,9 +3661,10 @@
       <x:c r="J94" s="49" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="K94" s="50" t="n">
+      <x:c r="K94" s="49" t="n">
         <x:v>27635</x:v>
       </x:c>
+      <x:c r="L94" s="58" t="str"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="46" t="str">
@@ -3585,9 +3693,10 @@
       <x:c r="J95" s="49" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="K95" s="50" t="n">
+      <x:c r="K95" s="49" t="n">
         <x:v>62680</x:v>
       </x:c>
+      <x:c r="L95" s="58" t="str"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="46" t="str">
@@ -3616,9 +3725,10 @@
       <x:c r="J96" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K96" s="50" t="n">
+      <x:c r="K96" s="49" t="n">
         <x:v>27738</x:v>
       </x:c>
+      <x:c r="L96" s="58" t="str"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="46" t="str">
@@ -3647,9 +3757,10 @@
       <x:c r="J97" s="49" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="K97" s="50" t="n">
+      <x:c r="K97" s="49" t="n">
         <x:v>14249</x:v>
       </x:c>
+      <x:c r="L97" s="58" t="str"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="46" t="str">
@@ -3678,9 +3789,10 @@
       <x:c r="J98" s="49" t="n">
         <x:v>194</x:v>
       </x:c>
-      <x:c r="K98" s="50" t="n">
+      <x:c r="K98" s="49" t="n">
         <x:v>240043</x:v>
       </x:c>
+      <x:c r="L98" s="58" t="str"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="46" t="str">
@@ -3709,9 +3821,10 @@
       <x:c r="J99" s="49" t="n">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="K99" s="50" t="n">
+      <x:c r="K99" s="49" t="n">
         <x:v>327452</x:v>
       </x:c>
+      <x:c r="L99" s="58" t="str"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="46" t="str">
@@ -3740,9 +3853,10 @@
       <x:c r="J100" s="49" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="K100" s="50" t="n">
+      <x:c r="K100" s="49" t="n">
         <x:v>87331</x:v>
       </x:c>
+      <x:c r="L100" s="58" t="str"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="46" t="str">
@@ -3771,9 +3885,10 @@
       <x:c r="J101" s="49" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="K101" s="50" t="n">
+      <x:c r="K101" s="49" t="n">
         <x:v>64682</x:v>
       </x:c>
+      <x:c r="L101" s="58" t="str"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="46" t="str">
@@ -3802,9 +3917,10 @@
       <x:c r="J102" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K102" s="50" t="n">
+      <x:c r="K102" s="49" t="n">
         <x:v>12960</x:v>
       </x:c>
+      <x:c r="L102" s="58" t="str"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="46" t="str">
@@ -3833,9 +3949,10 @@
       <x:c r="J103" s="49" t="n">
         <x:v>4050</x:v>
       </x:c>
-      <x:c r="K103" s="50" t="n">
+      <x:c r="K103" s="49" t="n">
         <x:v>2957527</x:v>
       </x:c>
+      <x:c r="L103" s="58" t="str"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="46" t="str">
@@ -3864,9 +3981,10 @@
       <x:c r="J104" s="49" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="K104" s="50" t="n">
+      <x:c r="K104" s="49" t="n">
         <x:v>15587</x:v>
       </x:c>
+      <x:c r="L104" s="58" t="str"/>
     </x:row>
     <x:row r="105">
       <x:c r="A105" s="46" t="str">
@@ -3895,9 +4013,10 @@
       <x:c r="J105" s="49" t="n">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="K105" s="50" t="n">
+      <x:c r="K105" s="49" t="n">
         <x:v>24409</x:v>
       </x:c>
+      <x:c r="L105" s="58" t="str"/>
     </x:row>
     <x:row r="106">
       <x:c r="A106" s="46" t="str">
@@ -3926,9 +4045,10 @@
       <x:c r="J106" s="49" t="n">
         <x:v>330</x:v>
       </x:c>
-      <x:c r="K106" s="50" t="n">
+      <x:c r="K106" s="49" t="n">
         <x:v>215447</x:v>
       </x:c>
+      <x:c r="L106" s="58" t="str"/>
     </x:row>
     <x:row r="107">
       <x:c r="A107" s="46" t="str">
@@ -3957,9 +4077,10 @@
       <x:c r="J107" s="49" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="K107" s="50" t="n">
+      <x:c r="K107" s="49" t="n">
         <x:v>91937</x:v>
       </x:c>
+      <x:c r="L107" s="58" t="str"/>
     </x:row>
     <x:row r="108">
       <x:c r="A108" s="46" t="str">
@@ -3988,9 +4109,10 @@
       <x:c r="J108" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K108" s="50" t="n">
+      <x:c r="K108" s="49" t="n">
         <x:v>47836</x:v>
       </x:c>
+      <x:c r="L108" s="58" t="str"/>
     </x:row>
     <x:row r="109">
       <x:c r="A109" s="46" t="str">
@@ -4019,9 +4141,10 @@
       <x:c r="J109" s="49" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="K109" s="50" t="n">
+      <x:c r="K109" s="49" t="n">
         <x:v>26435</x:v>
       </x:c>
+      <x:c r="L109" s="58" t="str"/>
     </x:row>
     <x:row r="110">
       <x:c r="A110" s="46" t="str">
@@ -4050,9 +4173,10 @@
       <x:c r="J110" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K110" s="50" t="n">
+      <x:c r="K110" s="49" t="n">
         <x:v>19085</x:v>
       </x:c>
+      <x:c r="L110" s="58" t="str"/>
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="46" t="str">
@@ -4081,9 +4205,10 @@
       <x:c r="J111" s="49" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="K111" s="50" t="n">
+      <x:c r="K111" s="49" t="n">
         <x:v>56289</x:v>
       </x:c>
+      <x:c r="L111" s="58" t="str"/>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="46" t="str">
@@ -4112,9 +4237,10 @@
       <x:c r="J112" s="49" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="K112" s="50" t="n">
+      <x:c r="K112" s="49" t="n">
         <x:v>65515</x:v>
       </x:c>
+      <x:c r="L112" s="58" t="str"/>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="46" t="str">
@@ -4143,9 +4269,10 @@
       <x:c r="J113" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K113" s="50" t="n">
+      <x:c r="K113" s="49" t="n">
         <x:v>65447</x:v>
       </x:c>
+      <x:c r="L113" s="58" t="str"/>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="46" t="str">
@@ -4174,9 +4301,10 @@
       <x:c r="J114" s="49" t="n">
         <x:v>203</x:v>
       </x:c>
-      <x:c r="K114" s="50" t="n">
+      <x:c r="K114" s="49" t="n">
         <x:v>106919</x:v>
       </x:c>
+      <x:c r="L114" s="58" t="str"/>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="46" t="str">
@@ -4205,9 +4333,10 @@
       <x:c r="J115" s="49" t="n">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="K115" s="50" t="n">
+      <x:c r="K115" s="49" t="n">
         <x:v>77953</x:v>
       </x:c>
+      <x:c r="L115" s="58" t="str"/>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="46" t="str">
@@ -4236,9 +4365,10 @@
       <x:c r="J116" s="49" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="K116" s="50" t="n">
+      <x:c r="K116" s="49" t="n">
         <x:v>46537</x:v>
       </x:c>
+      <x:c r="L116" s="58" t="str"/>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="46" t="str">
@@ -4267,9 +4397,10 @@
       <x:c r="J117" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K117" s="50" t="n">
+      <x:c r="K117" s="49" t="n">
         <x:v>31522</x:v>
       </x:c>
+      <x:c r="L117" s="58" t="str"/>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="41" t="str">
@@ -4294,9 +4425,10 @@
       <x:c r="J118" s="44" t="n">
         <x:v>932</x:v>
       </x:c>
-      <x:c r="K118" s="45" t="n">
+      <x:c r="K118" s="44" t="n">
         <x:v>494035</x:v>
       </x:c>
+      <x:c r="L118" s="57" t="str"/>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="46" t="str">
@@ -4325,9 +4457,10 @@
       <x:c r="J119" s="49" t="n">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="K119" s="50" t="n">
+      <x:c r="K119" s="49" t="n">
         <x:v>55989</x:v>
       </x:c>
+      <x:c r="L119" s="58" t="str"/>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="46" t="str">
@@ -4356,9 +4489,10 @@
       <x:c r="J120" s="49" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="K120" s="50" t="n">
+      <x:c r="K120" s="49" t="n">
         <x:v>56225</x:v>
       </x:c>
+      <x:c r="L120" s="58" t="str"/>
     </x:row>
     <x:row r="121">
       <x:c r="A121" s="46" t="str">
@@ -4387,9 +4521,10 @@
       <x:c r="J121" s="49" t="n">
         <x:v>538</x:v>
       </x:c>
-      <x:c r="K121" s="50" t="n">
+      <x:c r="K121" s="49" t="n">
         <x:v>228403</x:v>
       </x:c>
+      <x:c r="L121" s="58" t="str"/>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="46" t="str">
@@ -4418,9 +4553,10 @@
       <x:c r="J122" s="49" t="n">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="K122" s="50" t="n">
+      <x:c r="K122" s="49" t="n">
         <x:v>120764</x:v>
       </x:c>
+      <x:c r="L122" s="58" t="str"/>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="46" t="str">
@@ -4449,9 +4585,10 @@
       <x:c r="J123" s="49" t="n">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="K123" s="50" t="n">
+      <x:c r="K123" s="49" t="n">
         <x:v>14155</x:v>
       </x:c>
+      <x:c r="L123" s="58" t="str"/>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="46" t="str">
@@ -4480,9 +4617,10 @@
       <x:c r="J124" s="49" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K124" s="50" t="n">
+      <x:c r="K124" s="49" t="n">
         <x:v>18499</x:v>
       </x:c>
+      <x:c r="L124" s="58" t="str"/>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="41" t="str">
@@ -4503,7 +4641,8 @@
         <x:v>sin_dato</x:v>
       </x:c>
       <x:c r="J125" s="44"/>
-      <x:c r="K125" s="45"/>
+      <x:c r="K125" s="44"/>
+      <x:c r="L125" s="57" t="str"/>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="46" t="str">
@@ -4530,7 +4669,8 @@
       <x:c r="J126" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K126" s="50"/>
+      <x:c r="K126" s="49"/>
+      <x:c r="L126" s="58" t="str"/>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="41" t="str">
@@ -4555,9 +4695,10 @@
       <x:c r="J127" s="44" t="n">
         <x:v>1190</x:v>
       </x:c>
-      <x:c r="K127" s="45" t="n">
+      <x:c r="K127" s="44" t="n">
         <x:v>497438</x:v>
       </x:c>
+      <x:c r="L127" s="57" t="str"/>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="46" t="str">
@@ -4586,9 +4727,10 @@
       <x:c r="J128" s="49" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="K128" s="50" t="n">
+      <x:c r="K128" s="49" t="n">
         <x:v>26544</x:v>
       </x:c>
+      <x:c r="L128" s="58" t="str"/>
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="46" t="str">
@@ -4617,9 +4759,10 @@
       <x:c r="J129" s="49" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K129" s="50" t="n">
+      <x:c r="K129" s="49" t="n">
         <x:v>36192</x:v>
       </x:c>
+      <x:c r="L129" s="58" t="str"/>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="46" t="str">
@@ -4648,9 +4791,10 @@
       <x:c r="J130" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K130" s="50" t="n">
+      <x:c r="K130" s="49" t="n">
         <x:v>14721</x:v>
       </x:c>
+      <x:c r="L130" s="58" t="str"/>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="46" t="str">
@@ -4679,9 +4823,10 @@
       <x:c r="J131" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K131" s="50" t="n">
+      <x:c r="K131" s="49" t="n">
         <x:v>6908</x:v>
       </x:c>
+      <x:c r="L131" s="58" t="str"/>
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="46" t="str">
@@ -4710,9 +4855,10 @@
       <x:c r="J132" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K132" s="50" t="n">
+      <x:c r="K132" s="49" t="n">
         <x:v>14368</x:v>
       </x:c>
+      <x:c r="L132" s="58" t="str"/>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="46" t="str">
@@ -4741,9 +4887,10 @@
       <x:c r="J133" s="49" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="K133" s="50" t="n">
+      <x:c r="K133" s="49" t="n">
         <x:v>12436</x:v>
       </x:c>
+      <x:c r="L133" s="58" t="str"/>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="46" t="str">
@@ -4772,9 +4919,10 @@
       <x:c r="J134" s="49" t="n">
         <x:v>1058</x:v>
       </x:c>
-      <x:c r="K134" s="50" t="n">
+      <x:c r="K134" s="49" t="n">
         <x:v>257110</x:v>
       </x:c>
+      <x:c r="L134" s="58" t="str"/>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="46" t="str">
@@ -4803,9 +4951,10 @@
       <x:c r="J135" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K135" s="50" t="n">
+      <x:c r="K135" s="49" t="n">
         <x:v>18618</x:v>
       </x:c>
+      <x:c r="L135" s="58" t="str"/>
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="46" t="str">
@@ -4834,9 +4983,10 @@
       <x:c r="J136" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K136" s="50" t="n">
+      <x:c r="K136" s="49" t="n">
         <x:v>4165</x:v>
       </x:c>
+      <x:c r="L136" s="58" t="str"/>
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="46" t="str">
@@ -4865,9 +5015,10 @@
       <x:c r="J137" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K137" s="50" t="n">
+      <x:c r="K137" s="49" t="n">
         <x:v>23067</x:v>
       </x:c>
+      <x:c r="L137" s="58" t="str"/>
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="46" t="str">
@@ -4896,9 +5047,10 @@
       <x:c r="J138" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K138" s="50" t="n">
+      <x:c r="K138" s="49" t="n">
         <x:v>10887</x:v>
       </x:c>
+      <x:c r="L138" s="58" t="str"/>
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="46" t="str">
@@ -4927,9 +5079,10 @@
       <x:c r="J139" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K139" s="50" t="n">
+      <x:c r="K139" s="49" t="n">
         <x:v>16572</x:v>
       </x:c>
+      <x:c r="L139" s="58" t="str"/>
     </x:row>
     <x:row r="140">
       <x:c r="A140" s="46" t="str">
@@ -4958,9 +5111,10 @@
       <x:c r="J140" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K140" s="50" t="n">
+      <x:c r="K140" s="49" t="n">
         <x:v>3952</x:v>
       </x:c>
+      <x:c r="L140" s="58" t="str"/>
     </x:row>
     <x:row r="141">
       <x:c r="A141" s="46" t="str">
@@ -4989,9 +5143,10 @@
       <x:c r="J141" s="49" t="n">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="K141" s="50" t="n">
+      <x:c r="K141" s="49" t="n">
         <x:v>29744</x:v>
       </x:c>
+      <x:c r="L141" s="58" t="str"/>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="46" t="str">
@@ -5020,9 +5175,10 @@
       <x:c r="J142" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K142" s="50" t="n">
+      <x:c r="K142" s="49" t="n">
         <x:v>6957</x:v>
       </x:c>
+      <x:c r="L142" s="58" t="str"/>
     </x:row>
     <x:row r="143">
       <x:c r="A143" s="46" t="str">
@@ -5051,9 +5207,10 @@
       <x:c r="J143" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K143" s="50" t="n">
+      <x:c r="K143" s="49" t="n">
         <x:v>15197</x:v>
       </x:c>
+      <x:c r="L143" s="58" t="str"/>
     </x:row>
     <x:row r="144">
       <x:c r="A144" s="41" t="str">
@@ -5078,9 +5235,10 @@
       <x:c r="J144" s="44" t="n">
         <x:v>228</x:v>
       </x:c>
-      <x:c r="K144" s="45" t="n">
+      <x:c r="K144" s="44" t="n">
         <x:v>968660</x:v>
       </x:c>
+      <x:c r="L144" s="57" t="str"/>
     </x:row>
     <x:row r="145">
       <x:c r="A145" s="46" t="str">
@@ -5109,9 +5267,10 @@
       <x:c r="J145" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K145" s="50" t="n">
+      <x:c r="K145" s="49" t="n">
         <x:v>48034</x:v>
       </x:c>
+      <x:c r="L145" s="58" t="str"/>
     </x:row>
     <x:row r="146">
       <x:c r="A146" s="46" t="str">
@@ -5140,9 +5299,10 @@
       <x:c r="J146" s="49" t="n">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="K146" s="50" t="n">
+      <x:c r="K146" s="49" t="n">
         <x:v>191772</x:v>
       </x:c>
+      <x:c r="L146" s="58" t="str"/>
     </x:row>
     <x:row r="147">
       <x:c r="A147" s="46" t="str">
@@ -5171,9 +5331,10 @@
       <x:c r="J147" s="49" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="K147" s="50" t="n">
+      <x:c r="K147" s="49" t="n">
         <x:v>82607</x:v>
       </x:c>
+      <x:c r="L147" s="58" t="str"/>
     </x:row>
     <x:row r="148">
       <x:c r="A148" s="46" t="str">
@@ -5202,9 +5363,10 @@
       <x:c r="J148" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K148" s="50" t="n">
+      <x:c r="K148" s="49" t="n">
         <x:v>43955</x:v>
       </x:c>
+      <x:c r="L148" s="58" t="str"/>
     </x:row>
     <x:row r="149">
       <x:c r="A149" s="46" t="str">
@@ -5233,9 +5395,10 @@
       <x:c r="J149" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K149" s="50" t="n">
+      <x:c r="K149" s="49" t="n">
         <x:v>30147</x:v>
       </x:c>
+      <x:c r="L149" s="58" t="str"/>
     </x:row>
     <x:row r="150">
       <x:c r="A150" s="46" t="str">
@@ -5264,9 +5427,10 @@
       <x:c r="J150" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K150" s="50" t="n">
+      <x:c r="K150" s="49" t="n">
         <x:v>25775</x:v>
       </x:c>
+      <x:c r="L150" s="58" t="str"/>
     </x:row>
     <x:row r="151">
       <x:c r="A151" s="46" t="str">
@@ -5295,9 +5459,10 @@
       <x:c r="J151" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K151" s="50" t="n">
+      <x:c r="K151" s="49" t="n">
         <x:v>45370</x:v>
       </x:c>
+      <x:c r="L151" s="58" t="str"/>
     </x:row>
     <x:row r="152">
       <x:c r="A152" s="46" t="str">
@@ -5326,9 +5491,10 @@
       <x:c r="J152" s="49" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="K152" s="50" t="n">
+      <x:c r="K152" s="49" t="n">
         <x:v>224264</x:v>
       </x:c>
+      <x:c r="L152" s="58" t="str"/>
     </x:row>
     <x:row r="153">
       <x:c r="A153" s="46" t="str">
@@ -5357,9 +5523,10 @@
       <x:c r="J153" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K153" s="50" t="n">
+      <x:c r="K153" s="49" t="n">
         <x:v>20414</x:v>
       </x:c>
+      <x:c r="L153" s="58" t="str"/>
     </x:row>
     <x:row r="154">
       <x:c r="A154" s="46" t="str">
@@ -5388,9 +5555,10 @@
       <x:c r="J154" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K154" s="50" t="n">
+      <x:c r="K154" s="49" t="n">
         <x:v>35210</x:v>
       </x:c>
+      <x:c r="L154" s="58" t="str"/>
     </x:row>
     <x:row r="155">
       <x:c r="A155" s="46" t="str">
@@ -5419,9 +5587,10 @@
       <x:c r="J155" s="49" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="K155" s="50" t="n">
+      <x:c r="K155" s="49" t="n">
         <x:v>55584</x:v>
       </x:c>
+      <x:c r="L155" s="58" t="str"/>
     </x:row>
     <x:row r="156">
       <x:c r="A156" s="46" t="str">
@@ -5450,9 +5619,10 @@
       <x:c r="J156" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K156" s="50" t="n">
+      <x:c r="K156" s="49" t="n">
         <x:v>79279</x:v>
       </x:c>
+      <x:c r="L156" s="58" t="str"/>
     </x:row>
     <x:row r="157">
       <x:c r="A157" s="46" t="str">
@@ -5481,9 +5651,10 @@
       <x:c r="J157" s="49" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="K157" s="50" t="n">
+      <x:c r="K157" s="49" t="n">
         <x:v>86249</x:v>
       </x:c>
+      <x:c r="L157" s="58" t="str"/>
     </x:row>
     <x:row r="158">
       <x:c r="A158" s="41" t="str">
@@ -5508,9 +5679,10 @@
       <x:c r="J158" s="44" t="n">
         <x:v>1857</x:v>
       </x:c>
-      <x:c r="K158" s="45" t="n">
+      <x:c r="K158" s="44" t="n">
         <x:v>1699434</x:v>
       </x:c>
+      <x:c r="L158" s="57" t="str"/>
     </x:row>
     <x:row r="159">
       <x:c r="A159" s="46" t="str">
@@ -5539,9 +5711,10 @@
       <x:c r="J159" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K159" s="50" t="n">
+      <x:c r="K159" s="49" t="n">
         <x:v>32819</x:v>
       </x:c>
+      <x:c r="L159" s="58" t="str"/>
     </x:row>
     <x:row r="160">
       <x:c r="A160" s="46" t="str">
@@ -5570,9 +5743,10 @@
       <x:c r="J160" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K160" s="50" t="n">
+      <x:c r="K160" s="49" t="n">
         <x:v>45712</x:v>
       </x:c>
+      <x:c r="L160" s="58" t="str"/>
     </x:row>
     <x:row r="161">
       <x:c r="A161" s="46" t="str">
@@ -5601,9 +5775,10 @@
       <x:c r="J161" s="49" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="K161" s="50" t="n">
+      <x:c r="K161" s="49" t="n">
         <x:v>136646</x:v>
       </x:c>
+      <x:c r="L161" s="58" t="str"/>
     </x:row>
     <x:row r="162">
       <x:c r="A162" s="46" t="str">
@@ -5632,9 +5807,10 @@
       <x:c r="J162" s="49" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="K162" s="50" t="n">
+      <x:c r="K162" s="49" t="n">
         <x:v>131464</x:v>
       </x:c>
+      <x:c r="L162" s="58" t="str"/>
     </x:row>
     <x:row r="163">
       <x:c r="A163" s="46" t="str">
@@ -5663,9 +5839,10 @@
       <x:c r="J163" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K163" s="50" t="n">
+      <x:c r="K163" s="49" t="n">
         <x:v>29046</x:v>
       </x:c>
+      <x:c r="L163" s="58" t="str"/>
     </x:row>
     <x:row r="164">
       <x:c r="A164" s="46" t="str">
@@ -5694,9 +5871,10 @@
       <x:c r="J164" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K164" s="50" t="n">
+      <x:c r="K164" s="49" t="n">
         <x:v>17697</x:v>
       </x:c>
+      <x:c r="L164" s="58" t="str"/>
     </x:row>
     <x:row r="165">
       <x:c r="A165" s="46" t="str">
@@ -5725,9 +5903,10 @@
       <x:c r="J165" s="49" t="n">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="K165" s="50" t="n">
+      <x:c r="K165" s="49" t="n">
         <x:v>32223</x:v>
       </x:c>
+      <x:c r="L165" s="58" t="str"/>
     </x:row>
     <x:row r="166">
       <x:c r="A166" s="46" t="str">
@@ -5756,9 +5935,10 @@
       <x:c r="J166" s="49" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="K166" s="50" t="n">
+      <x:c r="K166" s="49" t="n">
         <x:v>82110</x:v>
       </x:c>
+      <x:c r="L166" s="58" t="str"/>
     </x:row>
     <x:row r="167">
       <x:c r="A167" s="46" t="str">
@@ -5787,9 +5967,10 @@
       <x:c r="J167" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K167" s="50" t="n">
+      <x:c r="K167" s="49" t="n">
         <x:v>23428</x:v>
       </x:c>
+      <x:c r="L167" s="58" t="str"/>
     </x:row>
     <x:row r="168">
       <x:c r="A168" s="46" t="str">
@@ -5818,9 +5999,10 @@
       <x:c r="J168" s="49" t="n">
         <x:v>1311</x:v>
       </x:c>
-      <x:c r="K168" s="50" t="n">
+      <x:c r="K168" s="49" t="n">
         <x:v>287759</x:v>
       </x:c>
+      <x:c r="L168" s="58" t="str"/>
     </x:row>
     <x:row r="169">
       <x:c r="A169" s="46" t="str">
@@ -5849,9 +6031,10 @@
       <x:c r="J169" s="49" t="n">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="K169" s="50" t="n">
+      <x:c r="K169" s="49" t="n">
         <x:v>106147</x:v>
       </x:c>
+      <x:c r="L169" s="58" t="str"/>
     </x:row>
     <x:row r="170">
       <x:c r="A170" s="46" t="str">
@@ -5880,9 +6063,10 @@
       <x:c r="J170" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K170" s="50" t="n">
+      <x:c r="K170" s="49" t="n">
         <x:v>10579</x:v>
       </x:c>
+      <x:c r="L170" s="58" t="str"/>
     </x:row>
     <x:row r="171">
       <x:c r="A171" s="46" t="str">
@@ -5911,9 +6095,10 @@
       <x:c r="J171" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K171" s="50" t="n">
+      <x:c r="K171" s="49" t="n">
         <x:v>44149</x:v>
       </x:c>
+      <x:c r="L171" s="58" t="str"/>
     </x:row>
     <x:row r="172">
       <x:c r="A172" s="46" t="str">
@@ -5942,9 +6127,10 @@
       <x:c r="J172" s="49" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="K172" s="50" t="n">
+      <x:c r="K172" s="49" t="n">
         <x:v>79428</x:v>
       </x:c>
+      <x:c r="L172" s="58" t="str"/>
     </x:row>
     <x:row r="173">
       <x:c r="A173" s="46" t="str">
@@ -5973,9 +6159,10 @@
       <x:c r="J173" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K173" s="50" t="n">
+      <x:c r="K173" s="49" t="n">
         <x:v>31958</x:v>
       </x:c>
+      <x:c r="L173" s="58" t="str"/>
     </x:row>
     <x:row r="174">
       <x:c r="A174" s="46" t="str">
@@ -6004,9 +6191,10 @@
       <x:c r="J174" s="49" t="n">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="K174" s="50" t="n">
+      <x:c r="K174" s="49" t="n">
         <x:v>342231</x:v>
       </x:c>
+      <x:c r="L174" s="58" t="str"/>
     </x:row>
     <x:row r="175">
       <x:c r="A175" s="46" t="str">
@@ -6035,9 +6223,10 @@
       <x:c r="J175" s="49" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K175" s="50" t="n">
+      <x:c r="K175" s="49" t="n">
         <x:v>27971</x:v>
       </x:c>
+      <x:c r="L175" s="58" t="str"/>
     </x:row>
     <x:row r="176">
       <x:c r="A176" s="46" t="str">
@@ -6066,9 +6255,10 @@
       <x:c r="J176" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K176" s="50" t="n">
+      <x:c r="K176" s="49" t="n">
         <x:v>45295</x:v>
       </x:c>
+      <x:c r="L176" s="58" t="str"/>
     </x:row>
     <x:row r="177">
       <x:c r="A177" s="46" t="str">
@@ -6097,9 +6287,10 @@
       <x:c r="J177" s="49" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="K177" s="50" t="n">
+      <x:c r="K177" s="49" t="n">
         <x:v>26333</x:v>
       </x:c>
+      <x:c r="L177" s="58" t="str"/>
     </x:row>
     <x:row r="178">
       <x:c r="A178" s="46" t="str">
@@ -6128,9 +6319,10 @@
       <x:c r="J178" s="49" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="K178" s="50" t="n">
+      <x:c r="K178" s="49" t="n">
         <x:v>53749</x:v>
       </x:c>
+      <x:c r="L178" s="58" t="str"/>
     </x:row>
     <x:row r="179">
       <x:c r="A179" s="46" t="str">
@@ -6159,9 +6351,10 @@
       <x:c r="J179" s="49" t="n">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="K179" s="50" t="n">
+      <x:c r="K179" s="49" t="n">
         <x:v>67831</x:v>
       </x:c>
+      <x:c r="L179" s="58" t="str"/>
     </x:row>
     <x:row r="180">
       <x:c r="A180" s="46" t="str">
@@ -6190,9 +6383,10 @@
       <x:c r="J180" s="49" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="K180" s="50" t="n">
+      <x:c r="K180" s="49" t="n">
         <x:v>44859</x:v>
       </x:c>
+      <x:c r="L180" s="58" t="str"/>
     </x:row>
     <x:row r="181">
       <x:c r="A181" s="41" t="str">
@@ -6217,9 +6411,10 @@
       <x:c r="J181" s="44" t="n">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="K181" s="45" t="n">
+      <x:c r="K181" s="44" t="n">
         <x:v>206327</x:v>
       </x:c>
+      <x:c r="L181" s="57" t="str"/>
     </x:row>
     <x:row r="182">
       <x:c r="A182" s="46" t="str">
@@ -6248,9 +6443,10 @@
       <x:c r="J182" s="49" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K182" s="50" t="n">
+      <x:c r="K182" s="49" t="n">
         <x:v>23155</x:v>
       </x:c>
+      <x:c r="L182" s="58" t="str"/>
     </x:row>
     <x:row r="183">
       <x:c r="A183" s="46" t="str">
@@ -6279,9 +6475,10 @@
       <x:c r="J183" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K183" s="50" t="n">
+      <x:c r="K183" s="49" t="n">
         <x:v>11781</x:v>
       </x:c>
+      <x:c r="L183" s="58" t="str"/>
     </x:row>
     <x:row r="184">
       <x:c r="A184" s="46" t="str">
@@ -6310,9 +6507,10 @@
       <x:c r="J184" s="49" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K184" s="50" t="n">
+      <x:c r="K184" s="49" t="n">
         <x:v>10150</x:v>
       </x:c>
+      <x:c r="L184" s="58" t="str"/>
     </x:row>
     <x:row r="185">
       <x:c r="A185" s="46" t="str">
@@ -6341,9 +6539,10 @@
       <x:c r="J185" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K185" s="50" t="n">
+      <x:c r="K185" s="49" t="n">
         <x:v>7922</x:v>
       </x:c>
+      <x:c r="L185" s="58" t="str"/>
     </x:row>
     <x:row r="186">
       <x:c r="A186" s="46" t="str">
@@ -6372,9 +6571,10 @@
       <x:c r="J186" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K186" s="50" t="n">
+      <x:c r="K186" s="49" t="n">
         <x:v>58843</x:v>
       </x:c>
+      <x:c r="L186" s="58" t="str"/>
     </x:row>
     <x:row r="187">
       <x:c r="A187" s="46" t="str">
@@ -6403,9 +6603,10 @@
       <x:c r="J187" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K187" s="50" t="n">
+      <x:c r="K187" s="49" t="n">
         <x:v>2380</x:v>
       </x:c>
+      <x:c r="L187" s="58" t="str"/>
     </x:row>
     <x:row r="188">
       <x:c r="A188" s="46" t="str">
@@ -6434,9 +6635,10 @@
       <x:c r="J188" s="49" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="K188" s="50" t="n">
+      <x:c r="K188" s="49" t="n">
         <x:v>12718</x:v>
       </x:c>
+      <x:c r="L188" s="58" t="str"/>
     </x:row>
     <x:row r="189">
       <x:c r="A189" s="46" t="str">
@@ -6465,9 +6667,10 @@
       <x:c r="J189" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K189" s="50" t="n">
+      <x:c r="K189" s="49" t="n">
         <x:v>4520</x:v>
       </x:c>
+      <x:c r="L189" s="58" t="str"/>
     </x:row>
     <x:row r="190">
       <x:c r="A190" s="46" t="str">
@@ -6496,9 +6699,10 @@
       <x:c r="J190" s="49" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K190" s="50" t="n">
+      <x:c r="K190" s="49" t="n">
         <x:v>9980</x:v>
       </x:c>
+      <x:c r="L190" s="58" t="str"/>
     </x:row>
     <x:row r="191">
       <x:c r="A191" s="46" t="str">
@@ -6525,7 +6729,8 @@
       <x:c r="J191" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K191" s="50"/>
+      <x:c r="K191" s="49"/>
+      <x:c r="L191" s="58" t="str"/>
     </x:row>
     <x:row r="192">
       <x:c r="A192" s="46" t="str">
@@ -6554,9 +6759,10 @@
       <x:c r="J192" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K192" s="50" t="n">
+      <x:c r="K192" s="49" t="n">
         <x:v>24610</x:v>
       </x:c>
+      <x:c r="L192" s="58" t="str"/>
     </x:row>
     <x:row r="193">
       <x:c r="A193" s="46" t="str">
@@ -6585,9 +6791,10 @@
       <x:c r="J193" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K193" s="50" t="n">
+      <x:c r="K193" s="49" t="n">
         <x:v>29997</x:v>
       </x:c>
+      <x:c r="L193" s="58" t="str"/>
     </x:row>
     <x:row r="194">
       <x:c r="A194" s="46" t="str">
@@ -6616,9 +6823,10 @@
       <x:c r="J194" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K194" s="50" t="n">
+      <x:c r="K194" s="49" t="n">
         <x:v>10271</x:v>
       </x:c>
+      <x:c r="L194" s="58" t="str"/>
     </x:row>
     <x:row r="195">
       <x:c r="A195" s="41" t="str">
@@ -6643,9 +6851,10 @@
       <x:c r="J195" s="44" t="n">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="K195" s="45" t="n">
+      <x:c r="K195" s="44" t="n">
         <x:v>138541</x:v>
       </x:c>
+      <x:c r="L195" s="57" t="str"/>
     </x:row>
     <x:row r="196">
       <x:c r="A196" s="46" t="str">
@@ -6674,9 +6883,10 @@
       <x:c r="J196" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K196" s="50" t="n">
+      <x:c r="K196" s="49" t="n">
         <x:v>32331</x:v>
       </x:c>
+      <x:c r="L196" s="58" t="str"/>
     </x:row>
     <x:row r="197">
       <x:c r="A197" s="46" t="str">
@@ -6705,9 +6915,10 @@
       <x:c r="J197" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K197" s="50" t="n">
+      <x:c r="K197" s="49" t="n">
         <x:v>4820</x:v>
       </x:c>
+      <x:c r="L197" s="58" t="str"/>
     </x:row>
     <x:row r="198">
       <x:c r="A198" s="46" t="str">
@@ -6736,9 +6947,10 @@
       <x:c r="J198" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K198" s="50" t="n">
+      <x:c r="K198" s="49" t="n">
         <x:v>9508</x:v>
       </x:c>
+      <x:c r="L198" s="58" t="str"/>
     </x:row>
     <x:row r="199">
       <x:c r="A199" s="46" t="str">
@@ -6767,9 +6979,10 @@
       <x:c r="J199" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K199" s="50" t="n">
+      <x:c r="K199" s="49" t="n">
         <x:v>6645</x:v>
       </x:c>
+      <x:c r="L199" s="58" t="str"/>
     </x:row>
     <x:row r="200">
       <x:c r="A200" s="46" t="str">
@@ -6798,9 +7011,10 @@
       <x:c r="J200" s="49" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="K200" s="50" t="n">
+      <x:c r="K200" s="49" t="n">
         <x:v>85237</x:v>
       </x:c>
+      <x:c r="L200" s="58" t="str"/>
     </x:row>
     <x:row r="201">
       <x:c r="A201" s="41" t="str">
@@ -6825,9 +7039,10 @@
       <x:c r="J201" s="44" t="n">
         <x:v>263</x:v>
       </x:c>
-      <x:c r="K201" s="45" t="n">
+      <x:c r="K201" s="44" t="n">
         <x:v>192831</x:v>
       </x:c>
+      <x:c r="L201" s="57" t="str"/>
     </x:row>
     <x:row r="202">
       <x:c r="A202" s="46" t="str">
@@ -6856,9 +7071,10 @@
       <x:c r="J202" s="49" t="n">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="K202" s="50" t="n">
+      <x:c r="K202" s="49" t="n">
         <x:v>7423</x:v>
       </x:c>
+      <x:c r="L202" s="58" t="str"/>
     </x:row>
     <x:row r="203">
       <x:c r="A203" s="46" t="str">
@@ -6887,9 +7103,10 @@
       <x:c r="J203" s="49" t="n">
         <x:v>156</x:v>
       </x:c>
-      <x:c r="K203" s="50" t="n">
+      <x:c r="K203" s="49" t="n">
         <x:v>100185</x:v>
       </x:c>
+      <x:c r="L203" s="58" t="str"/>
     </x:row>
     <x:row r="204">
       <x:c r="A204" s="46" t="str">
@@ -6918,9 +7135,10 @@
       <x:c r="J204" s="49" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K204" s="50" t="n">
+      <x:c r="K204" s="49" t="n">
         <x:v>55268</x:v>
       </x:c>
+      <x:c r="L204" s="58" t="str"/>
     </x:row>
     <x:row r="205">
       <x:c r="A205" s="46" t="str">
@@ -6949,9 +7167,10 @@
       <x:c r="J205" s="49" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="K205" s="50" t="n">
+      <x:c r="K205" s="49" t="n">
         <x:v>29955</x:v>
       </x:c>
+      <x:c r="L205" s="58" t="str"/>
     </x:row>
     <x:row r="206">
       <x:c r="A206" s="41" t="str">
@@ -6976,9 +7195,10 @@
       <x:c r="J206" s="44" t="n">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="K206" s="45" t="n">
+      <x:c r="K206" s="44" t="n">
         <x:v>119032</x:v>
       </x:c>
+      <x:c r="L206" s="57" t="str"/>
     </x:row>
     <x:row r="207">
       <x:c r="A207" s="46" t="str">
@@ -7007,9 +7227,10 @@
       <x:c r="J207" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K207" s="50" t="n">
+      <x:c r="K207" s="49" t="n">
         <x:v>10611</x:v>
       </x:c>
+      <x:c r="L207" s="58" t="str"/>
     </x:row>
     <x:row r="208">
       <x:c r="A208" s="46" t="str">
@@ -7038,9 +7259,10 @@
       <x:c r="J208" s="49" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="K208" s="50" t="n">
+      <x:c r="K208" s="49" t="n">
         <x:v>15745</x:v>
       </x:c>
+      <x:c r="L208" s="58" t="str"/>
     </x:row>
     <x:row r="209">
       <x:c r="A209" s="46" t="str">
@@ -7069,9 +7291,10 @@
       <x:c r="J209" s="49" t="n">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="K209" s="50" t="n">
+      <x:c r="K209" s="49" t="n">
         <x:v>87977</x:v>
       </x:c>
+      <x:c r="L209" s="58" t="str"/>
     </x:row>
     <x:row r="210">
       <x:c r="A210" s="46" t="str">
@@ -7100,9 +7323,10 @@
       <x:c r="J210" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K210" s="50" t="n">
+      <x:c r="K210" s="49" t="n">
         <x:v>4699</x:v>
       </x:c>
+      <x:c r="L210" s="58" t="str"/>
     </x:row>
     <x:row r="211">
       <x:c r="A211" s="41" t="str">
@@ -7127,9 +7351,10 @@
       <x:c r="J211" s="44" t="n">
         <x:v>21060</x:v>
       </x:c>
-      <x:c r="K211" s="45" t="n">
+      <x:c r="K211" s="44" t="n">
         <x:v>3272265</x:v>
       </x:c>
+      <x:c r="L211" s="57" t="str"/>
     </x:row>
     <x:row r="212">
       <x:c r="A212" s="46" t="str">
@@ -7158,9 +7383,10 @@
       <x:c r="J212" s="49" t="n">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="K212" s="50" t="n">
+      <x:c r="K212" s="49" t="n">
         <x:v>112454</x:v>
       </x:c>
+      <x:c r="L212" s="58" t="str"/>
     </x:row>
     <x:row r="213">
       <x:c r="A213" s="46" t="str">
@@ -7189,9 +7415,10 @@
       <x:c r="J213" s="49" t="n">
         <x:v>20466</x:v>
       </x:c>
-      <x:c r="K213" s="50" t="n">
+      <x:c r="K213" s="49" t="n">
         <x:v>2838174</x:v>
       </x:c>
+      <x:c r="L213" s="58" t="str"/>
     </x:row>
     <x:row r="214">
       <x:c r="A214" s="46" t="str">
@@ -7220,9 +7447,10 @@
       <x:c r="J214" s="49" t="n">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="K214" s="50" t="n">
+      <x:c r="K214" s="49" t="n">
         <x:v>107385</x:v>
       </x:c>
+      <x:c r="L214" s="58" t="str"/>
     </x:row>
     <x:row r="215">
       <x:c r="A215" s="46" t="str">
@@ -7251,9 +7479,10 @@
       <x:c r="J215" s="49" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="K215" s="50" t="n">
+      <x:c r="K215" s="49" t="n">
         <x:v>43238</x:v>
       </x:c>
+      <x:c r="L215" s="58" t="str"/>
     </x:row>
     <x:row r="216">
       <x:c r="A216" s="46" t="str">
@@ -7282,9 +7511,10 @@
       <x:c r="J216" s="49" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K216" s="50" t="n">
+      <x:c r="K216" s="49" t="n">
         <x:v>16520</x:v>
       </x:c>
+      <x:c r="L216" s="58" t="str"/>
     </x:row>
     <x:row r="217">
       <x:c r="A217" s="46" t="str">
@@ -7313,9 +7543,10 @@
       <x:c r="J217" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K217" s="50" t="n">
+      <x:c r="K217" s="49" t="n">
         <x:v>26844</x:v>
       </x:c>
+      <x:c r="L217" s="58" t="str"/>
     </x:row>
     <x:row r="218">
       <x:c r="A218" s="46" t="str">
@@ -7344,9 +7575,10 @@
       <x:c r="J218" s="49" t="n">
         <x:v>368</x:v>
       </x:c>
-      <x:c r="K218" s="50" t="n">
+      <x:c r="K218" s="49" t="n">
         <x:v>113409</x:v>
       </x:c>
+      <x:c r="L218" s="58" t="str"/>
     </x:row>
     <x:row r="219">
       <x:c r="A219" s="46" t="str">
@@ -7375,9 +7607,10 @@
       <x:c r="J219" s="49" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="K219" s="50" t="n">
+      <x:c r="K219" s="49" t="n">
         <x:v>14241</x:v>
       </x:c>
+      <x:c r="L219" s="58" t="str"/>
     </x:row>
     <x:row r="220">
       <x:c r="A220" s="41" t="str">
@@ -7402,9 +7635,10 @@
       <x:c r="J220" s="44" t="n">
         <x:v>305</x:v>
       </x:c>
-      <x:c r="K220" s="45" t="n">
+      <x:c r="K220" s="44" t="n">
         <x:v>403478</x:v>
       </x:c>
+      <x:c r="L220" s="57" t="str"/>
     </x:row>
     <x:row r="221">
       <x:c r="A221" s="46" t="str">
@@ -7433,9 +7667,10 @@
       <x:c r="J221" s="49" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="K221" s="50" t="n">
+      <x:c r="K221" s="49" t="n">
         <x:v>118177</x:v>
       </x:c>
+      <x:c r="L221" s="58" t="str"/>
     </x:row>
     <x:row r="222">
       <x:c r="A222" s="46" t="str">
@@ -7464,9 +7699,10 @@
       <x:c r="J222" s="49" t="n">
         <x:v>184</x:v>
       </x:c>
-      <x:c r="K222" s="50" t="n">
+      <x:c r="K222" s="49" t="n">
         <x:v>89454</x:v>
       </x:c>
+      <x:c r="L222" s="58" t="str"/>
     </x:row>
     <x:row r="223">
       <x:c r="A223" s="46" t="str">
@@ -7495,9 +7731,10 @@
       <x:c r="J223" s="49" t="n">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="K223" s="50" t="n">
+      <x:c r="K223" s="49" t="n">
         <x:v>195847</x:v>
       </x:c>
+      <x:c r="L223" s="58" t="str"/>
     </x:row>
     <x:row r="224">
       <x:c r="A224" s="41" t="str">
@@ -7522,9 +7759,10 @@
       <x:c r="J224" s="44" t="n">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="K224" s="45" t="n">
+      <x:c r="K224" s="44" t="n">
         <x:v>523524</x:v>
       </x:c>
+      <x:c r="L224" s="57" t="str"/>
     </x:row>
     <x:row r="225">
       <x:c r="A225" s="46" t="str">
@@ -7553,9 +7791,10 @@
       <x:c r="J225" s="49" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="K225" s="50" t="n">
+      <x:c r="K225" s="49" t="n">
         <x:v>56683</x:v>
       </x:c>
+      <x:c r="L225" s="58" t="str"/>
     </x:row>
     <x:row r="226">
       <x:c r="A226" s="46" t="str">
@@ -7584,9 +7823,10 @@
       <x:c r="J226" s="49" t="n">
         <x:v>441</x:v>
       </x:c>
-      <x:c r="K226" s="50" t="n">
+      <x:c r="K226" s="49" t="n">
         <x:v>466841</x:v>
       </x:c>
+      <x:c r="L226" s="58" t="str"/>
     </x:row>
     <x:row r="227">
       <x:c r="A227" s="41" t="str">
@@ -7611,9 +7851,10 @@
       <x:c r="J227" s="44" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="K227" s="45" t="n">
+      <x:c r="K227" s="44" t="n">
         <x:v>205253</x:v>
       </x:c>
+      <x:c r="L227" s="57" t="str"/>
     </x:row>
     <x:row r="228">
       <x:c r="A228" s="46" t="str">
@@ -7642,9 +7883,10 @@
       <x:c r="J228" s="49" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="K228" s="50" t="n">
+      <x:c r="K228" s="49" t="n">
         <x:v>11889</x:v>
       </x:c>
+      <x:c r="L228" s="58" t="str"/>
     </x:row>
     <x:row r="229">
       <x:c r="A229" s="46" t="str">
@@ -7673,9 +7915,10 @@
       <x:c r="J229" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K229" s="50" t="n">
+      <x:c r="K229" s="49" t="n">
         <x:v>9101</x:v>
       </x:c>
+      <x:c r="L229" s="58" t="str"/>
     </x:row>
     <x:row r="230">
       <x:c r="A230" s="46" t="str">
@@ -7704,9 +7947,10 @@
       <x:c r="J230" s="49" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="K230" s="50" t="n">
+      <x:c r="K230" s="49" t="n">
         <x:v>10645</x:v>
       </x:c>
+      <x:c r="L230" s="58" t="str"/>
     </x:row>
     <x:row r="231">
       <x:c r="A231" s="46" t="str">
@@ -7735,9 +7979,10 @@
       <x:c r="J231" s="49" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="K231" s="50" t="n">
+      <x:c r="K231" s="49" t="n">
         <x:v>108536</x:v>
       </x:c>
+      <x:c r="L231" s="58" t="str"/>
     </x:row>
     <x:row r="232">
       <x:c r="A232" s="46" t="str">
@@ -7766,9 +8011,10 @@
       <x:c r="J232" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K232" s="50" t="n">
+      <x:c r="K232" s="49" t="n">
         <x:v>9026</x:v>
       </x:c>
+      <x:c r="L232" s="58" t="str"/>
     </x:row>
     <x:row r="233">
       <x:c r="A233" s="46" t="str">
@@ -7797,9 +8043,10 @@
       <x:c r="J233" s="49" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="K233" s="50" t="n">
+      <x:c r="K233" s="49" t="n">
         <x:v>52902</x:v>
       </x:c>
+      <x:c r="L233" s="58" t="str"/>
     </x:row>
     <x:row r="234">
       <x:c r="A234" s="46" t="str">
@@ -7828,9 +8075,10 @@
       <x:c r="J234" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K234" s="50" t="n">
+      <x:c r="K234" s="49" t="n">
         <x:v>3154</x:v>
       </x:c>
+      <x:c r="L234" s="58" t="str"/>
     </x:row>
     <x:row r="235">
       <x:c r="A235" s="41" t="str">
@@ -7855,9 +8103,10 @@
       <x:c r="J235" s="44" t="n">
         <x:v>746</x:v>
       </x:c>
-      <x:c r="K235" s="45" t="n">
+      <x:c r="K235" s="44" t="n">
         <x:v>579082</x:v>
       </x:c>
+      <x:c r="L235" s="57" t="str"/>
     </x:row>
     <x:row r="236">
       <x:c r="A236" s="46" t="str">
@@ -7886,9 +8135,10 @@
       <x:c r="J236" s="49" t="n">
         <x:v>522</x:v>
       </x:c>
-      <x:c r="K236" s="50" t="n">
+      <x:c r="K236" s="49" t="n">
         <x:v>381116</x:v>
       </x:c>
+      <x:c r="L236" s="58" t="str"/>
     </x:row>
     <x:row r="237">
       <x:c r="A237" s="46" t="str">
@@ -7917,9 +8167,10 @@
       <x:c r="J237" s="49" t="n">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="K237" s="50" t="n">
+      <x:c r="K237" s="49" t="n">
         <x:v>22705</x:v>
       </x:c>
+      <x:c r="L237" s="58" t="str"/>
     </x:row>
     <x:row r="238">
       <x:c r="A238" s="46" t="str">
@@ -7948,9 +8199,10 @@
       <x:c r="J238" s="49" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="K238" s="50" t="n">
+      <x:c r="K238" s="49" t="n">
         <x:v>10906</x:v>
       </x:c>
+      <x:c r="L238" s="58" t="str"/>
     </x:row>
     <x:row r="239">
       <x:c r="A239" s="46" t="str">
@@ -7979,9 +8231,10 @@
       <x:c r="J239" s="49" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="K239" s="50" t="n">
+      <x:c r="K239" s="49" t="n">
         <x:v>7404</x:v>
       </x:c>
+      <x:c r="L239" s="58" t="str"/>
     </x:row>
     <x:row r="240">
       <x:c r="A240" s="46" t="str">
@@ -8010,9 +8263,10 @@
       <x:c r="J240" s="49" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="K240" s="50" t="n">
+      <x:c r="K240" s="49" t="n">
         <x:v>14078</x:v>
       </x:c>
+      <x:c r="L240" s="58" t="str"/>
     </x:row>
     <x:row r="241">
       <x:c r="A241" s="46" t="str">
@@ -8041,9 +8295,10 @@
       <x:c r="J241" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K241" s="50" t="n">
+      <x:c r="K241" s="49" t="n">
         <x:v>19404</x:v>
       </x:c>
+      <x:c r="L241" s="58" t="str"/>
     </x:row>
     <x:row r="242">
       <x:c r="A242" s="46" t="str">
@@ -8072,9 +8327,10 @@
       <x:c r="J242" s="49" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="K242" s="50" t="n">
+      <x:c r="K242" s="49" t="n">
         <x:v>65726</x:v>
       </x:c>
+      <x:c r="L242" s="58" t="str"/>
     </x:row>
     <x:row r="243">
       <x:c r="A243" s="46" t="str">
@@ -8103,9 +8359,10 @@
       <x:c r="J243" s="49" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="K243" s="50" t="n">
+      <x:c r="K243" s="49" t="n">
         <x:v>43541</x:v>
       </x:c>
+      <x:c r="L243" s="58" t="str"/>
     </x:row>
     <x:row r="244">
       <x:c r="A244" s="46" t="str">
@@ -8134,9 +8391,10 @@
       <x:c r="J244" s="49" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="K244" s="50" t="n">
+      <x:c r="K244" s="49" t="n">
         <x:v>14202</x:v>
       </x:c>
+      <x:c r="L244" s="58" t="str"/>
     </x:row>
     <x:row r="245">
       <x:c r="A245" s="41" t="str">
@@ -8161,9 +8419,10 @@
       <x:c r="J245" s="44" t="n">
         <x:v>172</x:v>
       </x:c>
-      <x:c r="K245" s="45" t="n">
+      <x:c r="K245" s="44" t="n">
         <x:v>117650</x:v>
       </x:c>
+      <x:c r="L245" s="57" t="str"/>
     </x:row>
     <x:row r="246">
       <x:c r="A246" s="46" t="str">
@@ -8192,9 +8451,10 @@
       <x:c r="J246" s="49" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="K246" s="50" t="n">
+      <x:c r="K246" s="49" t="n">
         <x:v>8167</x:v>
       </x:c>
+      <x:c r="L246" s="58" t="str"/>
     </x:row>
     <x:row r="247">
       <x:c r="A247" s="46" t="str">
@@ -8223,9 +8483,10 @@
       <x:c r="J247" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K247" s="50" t="n">
+      <x:c r="K247" s="49" t="n">
         <x:v>10871</x:v>
       </x:c>
+      <x:c r="L247" s="58" t="str"/>
     </x:row>
     <x:row r="248">
       <x:c r="A248" s="46" t="str">
@@ -8254,9 +8515,10 @@
       <x:c r="J248" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K248" s="50" t="n">
+      <x:c r="K248" s="49" t="n">
         <x:v>14048</x:v>
       </x:c>
+      <x:c r="L248" s="58" t="str"/>
     </x:row>
     <x:row r="249">
       <x:c r="A249" s="46" t="str">
@@ -8285,9 +8547,10 @@
       <x:c r="J249" s="49" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K249" s="50" t="n">
+      <x:c r="K249" s="49" t="n">
         <x:v>7118</x:v>
       </x:c>
+      <x:c r="L249" s="58" t="str"/>
     </x:row>
     <x:row r="250">
       <x:c r="A250" s="46" t="str">
@@ -8316,9 +8579,10 @@
       <x:c r="J250" s="49" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="K250" s="50" t="n">
+      <x:c r="K250" s="49" t="n">
         <x:v>9098</x:v>
       </x:c>
+      <x:c r="L250" s="58" t="str"/>
     </x:row>
     <x:row r="251">
       <x:c r="A251" s="46" t="str">
@@ -8347,9 +8611,10 @@
       <x:c r="J251" s="49" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="K251" s="50" t="n">
+      <x:c r="K251" s="49" t="n">
         <x:v>5194</x:v>
       </x:c>
+      <x:c r="L251" s="58" t="str"/>
     </x:row>
     <x:row r="252">
       <x:c r="A252" s="46" t="str">
@@ -8378,9 +8643,10 @@
       <x:c r="J252" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="K252" s="50" t="n">
+      <x:c r="K252" s="49" t="n">
         <x:v>6584</x:v>
       </x:c>
+      <x:c r="L252" s="58" t="str"/>
     </x:row>
     <x:row r="253">
       <x:c r="A253" s="46" t="str">
@@ -8409,9 +8675,10 @@
       <x:c r="J253" s="49" t="n">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="K253" s="50" t="n">
+      <x:c r="K253" s="49" t="n">
         <x:v>24801</x:v>
       </x:c>
+      <x:c r="L253" s="58" t="str"/>
     </x:row>
     <x:row r="254">
       <x:c r="A254" s="46" t="str">
@@ -8440,9 +8707,10 @@
       <x:c r="J254" s="49" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="K254" s="50" t="n">
+      <x:c r="K254" s="49" t="n">
         <x:v>31769</x:v>
       </x:c>
+      <x:c r="L254" s="58" t="str"/>
     </x:row>
     <x:row r="255">
       <x:c r="A255" s="41" t="str">
@@ -8463,7 +8731,8 @@
         <x:v>sin_dato</x:v>
       </x:c>
       <x:c r="J255" s="44"/>
-      <x:c r="K255" s="45"/>
+      <x:c r="K255" s="44"/>
+      <x:c r="L255" s="57" t="str"/>
     </x:row>
     <x:row r="256">
       <x:c r="A256" s="51" t="str">
@@ -8490,12 +8759,13 @@
       <x:c r="J256" s="54" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K256" s="55"/>
+      <x:c r="K256" s="54"/>
+      <x:c r="L256" s="59" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:K2"/>
-    <x:mergeCell ref="A3:K3"/>
+    <x:mergeCell ref="A1:L2"/>
+    <x:mergeCell ref="A3:L3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>